<commit_message>
Pull monthly active developers from Open Dev Data
Artemis exposes developer metrics only for Ethereum and its API is paid,
so developers now come from Electric Capital's Open Dev Data snapshot
(eco_mads, CC BY 4.0, no key). The parquet file is cached per snapshot
version. exclusive_devs is the default because all_devs is inflated for
EVM chains by shared multichain repos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G864rZBoCAcVfxiVNuU5Yp
</commit_message>
<xml_diff>
--- a/crypto_compare/output/l1_comparison.xlsx
+++ b/crypto_compare/output/l1_comparison.xlsx
@@ -279,7 +279,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -414,9 +414,6 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -489,8 +486,8 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -641,6 +638,12 @@
 комиссии за 365 дн (Ethereum)</t>
       </text>
     </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -681,6 +684,12 @@
 комиссии за 365 дн (Solana)</t>
       </text>
     </comment>
+    <comment ref="J6" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -721,6 +730,12 @@
 комиссии за 365 дн (Sui)</t>
       </text>
     </comment>
+    <comment ref="J7" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -761,6 +776,12 @@
 комиссии за 365 дн (Aptos)</t>
       </text>
     </comment>
+    <comment ref="J8" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C9" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -801,6 +822,12 @@
 комиссии за 365 дн (Avalanche)</t>
       </text>
     </comment>
+    <comment ref="J9" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C10" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -841,6 +868,12 @@
 комиссии за 365 дн (Near)</t>
       </text>
     </comment>
+    <comment ref="J10" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C11" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -881,6 +914,12 @@
 комиссии за 365 дн (TON)</t>
       </text>
     </comment>
+    <comment ref="J11" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C12" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -921,6 +960,12 @@
 комиссии за 365 дн (Tron)</t>
       </text>
     </comment>
+    <comment ref="J12" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+      </text>
+    </comment>
     <comment ref="C13" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -961,6 +1006,12 @@
 комиссии за 365 дн (Hyperliquid)</t>
       </text>
     </comment>
+    <comment ref="J13" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0. ⚠ за 6 мес 24 → 4: скачок больше чем в 5 раз, часто это перепривязка общих репозиториев к сети, а не реальный приток разработчиков</t>
+      </text>
+    </comment>
     <comment ref="C14" authorId="0" shapeId="0">
       <text>
         <t>CoinGecko, 30.09.2026</t>
@@ -999,6 +1050,12 @@
       <text>
         <t>DeFiLlama, 30.09.2026
 комиссии за 365 дн (Monad)</t>
+      </text>
+    </comment>
+    <comment ref="J14" authorId="0" shapeId="0">
+      <text>
+        <t>Open Dev Data, 30.09.2026
+exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
       </text>
     </comment>
   </commentList>
@@ -1397,13 +1454,13 @@
         </is>
       </c>
       <c r="C5" s="44" t="n">
-        <v>327258.690254</v>
+        <v>327944.680337</v>
       </c>
       <c r="D5" s="44" t="n">
-        <v>327258.690254</v>
+        <v>327944.680337</v>
       </c>
       <c r="E5" s="44" t="n">
-        <v>53918.369868</v>
+        <v>53303.04256</v>
       </c>
       <c r="F5" s="44" t="n">
         <v>53909.531522</v>
@@ -1417,34 +1474,36 @@
       <c r="I5" s="45" t="n">
         <v>202.689948</v>
       </c>
-      <c r="J5" s="46" t="n"/>
-      <c r="K5" s="47" t="n"/>
-      <c r="L5" s="48" t="n"/>
-      <c r="M5" s="49">
+      <c r="J5" s="44" t="n">
+        <v>3270</v>
+      </c>
+      <c r="K5" s="46" t="n"/>
+      <c r="L5" s="47" t="n"/>
+      <c r="M5" s="48">
         <f>IF(OR(E5="",F5="",F5=0),"",E5/F5-1)</f>
         <v/>
       </c>
-      <c r="N5" s="49">
+      <c r="N5" s="48">
         <f>IF(OR(G5="",H5="",H5=0),"",G5/H5-1)</f>
         <v/>
       </c>
-      <c r="O5" s="50">
+      <c r="O5" s="49">
         <f>IF(OR(C5="",E5="",E5=0),"",C5/E5)</f>
         <v/>
       </c>
-      <c r="P5" s="51">
+      <c r="P5" s="50">
         <f>IF(OR(C5="",I5="",I5=0),"",C5/I5)</f>
         <v/>
       </c>
-      <c r="Q5" s="50">
+      <c r="Q5" s="49">
         <f>IF(OR(C5="",D5="",C5=0),"",D5/C5)</f>
         <v/>
       </c>
-      <c r="R5" s="52">
+      <c r="R5" s="51">
         <f>Расчёт!K5</f>
         <v/>
       </c>
-      <c r="S5" s="52">
+      <c r="S5" s="51">
         <f>IF(R5="","",RANK(R5,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1461,13 +1520,13 @@
         </is>
       </c>
       <c r="C6" s="44" t="n">
-        <v>69988.26169699999</v>
+        <v>70355.204557</v>
       </c>
       <c r="D6" s="44" t="n">
-        <v>75581.369252</v>
+        <v>75977.633946</v>
       </c>
       <c r="E6" s="44" t="n">
-        <v>6471.36886</v>
+        <v>6568.178533</v>
       </c>
       <c r="F6" s="44" t="n">
         <v>6357.767767</v>
@@ -1481,34 +1540,36 @@
       <c r="I6" s="45" t="n">
         <v>239.426752</v>
       </c>
-      <c r="J6" s="46" t="n"/>
-      <c r="K6" s="47" t="n"/>
-      <c r="L6" s="48" t="n"/>
-      <c r="M6" s="49">
+      <c r="J6" s="44" t="n">
+        <v>1080</v>
+      </c>
+      <c r="K6" s="46" t="n"/>
+      <c r="L6" s="47" t="n"/>
+      <c r="M6" s="48">
         <f>IF(OR(E6="",F6="",F6=0),"",E6/F6-1)</f>
         <v/>
       </c>
-      <c r="N6" s="49">
+      <c r="N6" s="48">
         <f>IF(OR(G6="",H6="",H6=0),"",G6/H6-1)</f>
         <v/>
       </c>
-      <c r="O6" s="50">
+      <c r="O6" s="49">
         <f>IF(OR(C6="",E6="",E6=0),"",C6/E6)</f>
         <v/>
       </c>
-      <c r="P6" s="51">
+      <c r="P6" s="50">
         <f>IF(OR(C6="",I6="",I6=0),"",C6/I6)</f>
         <v/>
       </c>
-      <c r="Q6" s="50">
+      <c r="Q6" s="49">
         <f>IF(OR(C6="",D6="",C6=0),"",D6/C6)</f>
         <v/>
       </c>
-      <c r="R6" s="52">
+      <c r="R6" s="51">
         <f>Расчёт!K6</f>
         <v/>
       </c>
-      <c r="S6" s="52">
+      <c r="S6" s="51">
         <f>IF(R6="","",RANK(R6,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1525,13 +1586,13 @@
         </is>
       </c>
       <c r="C7" s="44" t="n">
-        <v>4767.521283</v>
+        <v>4865.721245</v>
       </c>
       <c r="D7" s="44" t="n">
-        <v>11637.930067</v>
+        <v>11877.644633</v>
       </c>
       <c r="E7" s="44" t="n">
-        <v>559.329125</v>
+        <v>551.750347</v>
       </c>
       <c r="F7" s="44" t="n">
         <v>570.720387</v>
@@ -1545,34 +1606,36 @@
       <c r="I7" s="45" t="n">
         <v>3.512066</v>
       </c>
-      <c r="J7" s="46" t="n"/>
-      <c r="K7" s="47" t="n"/>
-      <c r="L7" s="48" t="n"/>
-      <c r="M7" s="49">
+      <c r="J7" s="44" t="n">
+        <v>254</v>
+      </c>
+      <c r="K7" s="46" t="n"/>
+      <c r="L7" s="47" t="n"/>
+      <c r="M7" s="48">
         <f>IF(OR(E7="",F7="",F7=0),"",E7/F7-1)</f>
         <v/>
       </c>
-      <c r="N7" s="49">
+      <c r="N7" s="48">
         <f>IF(OR(G7="",H7="",H7=0),"",G7/H7-1)</f>
         <v/>
       </c>
-      <c r="O7" s="50">
+      <c r="O7" s="49">
         <f>IF(OR(C7="",E7="",E7=0),"",C7/E7)</f>
         <v/>
       </c>
-      <c r="P7" s="51">
+      <c r="P7" s="50">
         <f>IF(OR(C7="",I7="",I7=0),"",C7/I7)</f>
         <v/>
       </c>
-      <c r="Q7" s="50">
+      <c r="Q7" s="49">
         <f>IF(OR(C7="",D7="",C7=0),"",D7/C7)</f>
         <v/>
       </c>
-      <c r="R7" s="52">
+      <c r="R7" s="51">
         <f>Расчёт!K7</f>
         <v/>
       </c>
-      <c r="S7" s="52">
+      <c r="S7" s="51">
         <f>IF(R7="","",RANK(R7,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1589,18 +1652,18 @@
         </is>
       </c>
       <c r="C8" s="44" t="n">
-        <v>687.9191049999999</v>
+        <v>690.49137</v>
       </c>
       <c r="D8" s="44" t="n">
-        <v>955.210046</v>
+        <v>958.7853270000001</v>
       </c>
       <c r="E8" s="44" t="n">
-        <v>55.740282</v>
+        <v>55.53995</v>
       </c>
       <c r="F8" s="44" t="n">
         <v>285.748159</v>
       </c>
-      <c r="G8" s="53" t="n">
+      <c r="G8" s="52" t="n">
         <v>35921</v>
       </c>
       <c r="H8" s="44" t="n">
@@ -1609,34 +1672,36 @@
       <c r="I8" s="45" t="n">
         <v>1.145126</v>
       </c>
-      <c r="J8" s="46" t="n"/>
-      <c r="K8" s="47" t="n"/>
-      <c r="L8" s="48" t="n"/>
-      <c r="M8" s="49">
+      <c r="J8" s="44" t="n">
+        <v>92</v>
+      </c>
+      <c r="K8" s="46" t="n"/>
+      <c r="L8" s="47" t="n"/>
+      <c r="M8" s="48">
         <f>IF(OR(E8="",F8="",F8=0),"",E8/F8-1)</f>
         <v/>
       </c>
-      <c r="N8" s="49">
+      <c r="N8" s="48">
         <f>IF(OR(G8="",H8="",H8=0),"",G8/H8-1)</f>
         <v/>
       </c>
-      <c r="O8" s="50">
+      <c r="O8" s="49">
         <f>IF(OR(C8="",E8="",E8=0),"",C8/E8)</f>
         <v/>
       </c>
-      <c r="P8" s="51">
+      <c r="P8" s="50">
         <f>IF(OR(C8="",I8="",I8=0),"",C8/I8)</f>
         <v/>
       </c>
-      <c r="Q8" s="50">
+      <c r="Q8" s="49">
         <f>IF(OR(C8="",D8="",C8=0),"",D8/C8)</f>
         <v/>
       </c>
-      <c r="R8" s="52">
+      <c r="R8" s="51">
         <f>Расчёт!K8</f>
         <v/>
       </c>
-      <c r="S8" s="52">
+      <c r="S8" s="51">
         <f>IF(R8="","",RANK(R8,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1653,54 +1718,56 @@
         </is>
       </c>
       <c r="C9" s="44" t="n">
-        <v>4829.34046</v>
+        <v>4879.641119</v>
       </c>
       <c r="D9" s="44" t="n">
-        <v>5120.001442</v>
+        <v>5173.313795</v>
       </c>
       <c r="E9" s="44" t="n">
-        <v>640.767554</v>
+        <v>626.279733</v>
       </c>
       <c r="F9" s="44" t="n">
         <v>724.301796</v>
       </c>
-      <c r="G9" s="53" t="n">
+      <c r="G9" s="52" t="n">
         <v>21091</v>
       </c>
-      <c r="H9" s="53" t="n">
+      <c r="H9" s="52" t="n">
         <v>643627</v>
       </c>
       <c r="I9" s="45" t="n">
         <v>4.076565</v>
       </c>
-      <c r="J9" s="46" t="n"/>
-      <c r="K9" s="47" t="n"/>
-      <c r="L9" s="48" t="n"/>
-      <c r="M9" s="49">
+      <c r="J9" s="44" t="n">
+        <v>108</v>
+      </c>
+      <c r="K9" s="46" t="n"/>
+      <c r="L9" s="47" t="n"/>
+      <c r="M9" s="48">
         <f>IF(OR(E9="",F9="",F9=0),"",E9/F9-1)</f>
         <v/>
       </c>
-      <c r="N9" s="49">
+      <c r="N9" s="48">
         <f>IF(OR(G9="",H9="",H9=0),"",G9/H9-1)</f>
         <v/>
       </c>
-      <c r="O9" s="50">
+      <c r="O9" s="49">
         <f>IF(OR(C9="",E9="",E9=0),"",C9/E9)</f>
         <v/>
       </c>
-      <c r="P9" s="51">
+      <c r="P9" s="50">
         <f>IF(OR(C9="",I9="",I9=0),"",C9/I9)</f>
         <v/>
       </c>
-      <c r="Q9" s="50">
+      <c r="Q9" s="49">
         <f>IF(OR(C9="",D9="",C9=0),"",D9/C9)</f>
         <v/>
       </c>
-      <c r="R9" s="52">
+      <c r="R9" s="51">
         <f>Расчёт!K9</f>
         <v/>
       </c>
-      <c r="S9" s="52">
+      <c r="S9" s="51">
         <f>IF(R9="","",RANK(R9,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1717,54 +1784,56 @@
         </is>
       </c>
       <c r="C10" s="44" t="n">
-        <v>6908.777867</v>
+        <v>7048.836656</v>
       </c>
       <c r="D10" s="44" t="n">
-        <v>6908.778987</v>
+        <v>7048.837611</v>
       </c>
       <c r="E10" s="44" t="n">
-        <v>239.929727</v>
+        <v>236.616937</v>
       </c>
       <c r="F10" s="44" t="n">
         <v>95.21909100000001</v>
       </c>
-      <c r="G10" s="53" t="n">
+      <c r="G10" s="52" t="n">
         <v>76790</v>
       </c>
-      <c r="H10" s="53" t="n">
+      <c r="H10" s="52" t="n">
         <v>3067142</v>
       </c>
       <c r="I10" s="45" t="n">
         <v>1.261909</v>
       </c>
-      <c r="J10" s="46" t="n"/>
-      <c r="K10" s="47" t="n"/>
-      <c r="L10" s="48" t="n"/>
-      <c r="M10" s="49">
+      <c r="J10" s="44" t="n">
+        <v>150</v>
+      </c>
+      <c r="K10" s="46" t="n"/>
+      <c r="L10" s="47" t="n"/>
+      <c r="M10" s="48">
         <f>IF(OR(E10="",F10="",F10=0),"",E10/F10-1)</f>
         <v/>
       </c>
-      <c r="N10" s="49">
+      <c r="N10" s="48">
         <f>IF(OR(G10="",H10="",H10=0),"",G10/H10-1)</f>
         <v/>
       </c>
-      <c r="O10" s="50">
+      <c r="O10" s="49">
         <f>IF(OR(C10="",E10="",E10=0),"",C10/E10)</f>
         <v/>
       </c>
-      <c r="P10" s="51">
+      <c r="P10" s="50">
         <f>IF(OR(C10="",I10="",I10=0),"",C10/I10)</f>
         <v/>
       </c>
-      <c r="Q10" s="50">
+      <c r="Q10" s="49">
         <f>IF(OR(C10="",D10="",C10=0),"",D10/C10)</f>
         <v/>
       </c>
-      <c r="R10" s="52">
+      <c r="R10" s="51">
         <f>Расчёт!K10</f>
         <v/>
       </c>
-      <c r="S10" s="52">
+      <c r="S10" s="51">
         <f>IF(R10="","",RANK(R10,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1781,13 +1850,13 @@
         </is>
       </c>
       <c r="C11" s="44" t="n">
-        <v>4228.799095</v>
+        <v>4238.049641</v>
       </c>
       <c r="D11" s="44" t="n">
-        <v>7895.284465</v>
+        <v>7912.528129</v>
       </c>
       <c r="E11" s="44" t="n">
-        <v>55.149255</v>
+        <v>54.352401</v>
       </c>
       <c r="F11" s="44" t="n">
         <v>55.174661</v>
@@ -1801,34 +1870,36 @@
       <c r="I11" s="45" t="n">
         <v>2.119862</v>
       </c>
-      <c r="J11" s="46" t="n"/>
-      <c r="K11" s="47" t="n"/>
-      <c r="L11" s="48" t="n"/>
-      <c r="M11" s="49">
+      <c r="J11" s="44" t="n">
+        <v>191</v>
+      </c>
+      <c r="K11" s="46" t="n"/>
+      <c r="L11" s="47" t="n"/>
+      <c r="M11" s="48">
         <f>IF(OR(E11="",F11="",F11=0),"",E11/F11-1)</f>
         <v/>
       </c>
-      <c r="N11" s="49">
+      <c r="N11" s="48">
         <f>IF(OR(G11="",H11="",H11=0),"",G11/H11-1)</f>
         <v/>
       </c>
-      <c r="O11" s="50">
+      <c r="O11" s="49">
         <f>IF(OR(C11="",E11="",E11=0),"",C11/E11)</f>
         <v/>
       </c>
-      <c r="P11" s="51">
+      <c r="P11" s="50">
         <f>IF(OR(C11="",I11="",I11=0),"",C11/I11)</f>
         <v/>
       </c>
-      <c r="Q11" s="50">
+      <c r="Q11" s="49">
         <f>IF(OR(C11="",D11="",C11=0),"",D11/C11)</f>
         <v/>
       </c>
-      <c r="R11" s="52">
+      <c r="R11" s="51">
         <f>Расчёт!K11</f>
         <v/>
       </c>
-      <c r="S11" s="52">
+      <c r="S11" s="51">
         <f>IF(R11="","",RANK(R11,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1845,13 +1916,13 @@
         </is>
       </c>
       <c r="C12" s="44" t="n">
-        <v>32174.288951</v>
+        <v>32097.231712</v>
       </c>
       <c r="D12" s="44" t="n">
-        <v>32174.313939</v>
+        <v>32097.240025</v>
       </c>
       <c r="E12" s="44" t="n">
-        <v>5678.20312</v>
+        <v>5638.408003</v>
       </c>
       <c r="F12" s="44" t="n">
         <v>4797.537404</v>
@@ -1865,34 +1936,36 @@
       <c r="I12" s="45" t="n">
         <v>348.971536</v>
       </c>
-      <c r="J12" s="46" t="n"/>
-      <c r="K12" s="47" t="n"/>
-      <c r="L12" s="48" t="n"/>
-      <c r="M12" s="49">
+      <c r="J12" s="44" t="n">
+        <v>70</v>
+      </c>
+      <c r="K12" s="46" t="n"/>
+      <c r="L12" s="47" t="n"/>
+      <c r="M12" s="48">
         <f>IF(OR(E12="",F12="",F12=0),"",E12/F12-1)</f>
         <v/>
       </c>
-      <c r="N12" s="49">
+      <c r="N12" s="48">
         <f>IF(OR(G12="",H12="",H12=0),"",G12/H12-1)</f>
         <v/>
       </c>
-      <c r="O12" s="50">
+      <c r="O12" s="49">
         <f>IF(OR(C12="",E12="",E12=0),"",C12/E12)</f>
         <v/>
       </c>
-      <c r="P12" s="51">
+      <c r="P12" s="50">
         <f>IF(OR(C12="",I12="",I12=0),"",C12/I12)</f>
         <v/>
       </c>
-      <c r="Q12" s="50">
+      <c r="Q12" s="49">
         <f>IF(OR(C12="",D12="",C12=0),"",D12/C12)</f>
         <v/>
       </c>
-      <c r="R12" s="52">
+      <c r="R12" s="51">
         <f>Расчёт!K12</f>
         <v/>
       </c>
-      <c r="S12" s="52">
+      <c r="S12" s="51">
         <f>IF(R12="","",RANK(R12,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1909,13 +1982,13 @@
         </is>
       </c>
       <c r="C13" s="44" t="n">
-        <v>19075.239849</v>
+        <v>19786.883821</v>
       </c>
       <c r="D13" s="44" t="n">
-        <v>81919.814663</v>
+        <v>84976.014364</v>
       </c>
       <c r="E13" s="44" t="n">
-        <v>1190.593415</v>
+        <v>1171.952848</v>
       </c>
       <c r="F13" s="44" t="n">
         <v>1672.171573</v>
@@ -1929,34 +2002,36 @@
       <c r="I13" s="45" t="n">
         <v>910.588444</v>
       </c>
-      <c r="J13" s="46" t="n"/>
-      <c r="K13" s="47" t="n"/>
-      <c r="L13" s="48" t="n"/>
-      <c r="M13" s="49">
+      <c r="J13" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" s="46" t="n"/>
+      <c r="L13" s="47" t="n"/>
+      <c r="M13" s="48">
         <f>IF(OR(E13="",F13="",F13=0),"",E13/F13-1)</f>
         <v/>
       </c>
-      <c r="N13" s="49">
+      <c r="N13" s="48">
         <f>IF(OR(G13="",H13="",H13=0),"",G13/H13-1)</f>
         <v/>
       </c>
-      <c r="O13" s="50">
+      <c r="O13" s="49">
         <f>IF(OR(C13="",E13="",E13=0),"",C13/E13)</f>
         <v/>
       </c>
-      <c r="P13" s="51">
+      <c r="P13" s="50">
         <f>IF(OR(C13="",I13="",I13=0),"",C13/I13)</f>
         <v/>
       </c>
-      <c r="Q13" s="50">
+      <c r="Q13" s="49">
         <f>IF(OR(C13="",D13="",C13=0),"",D13/C13)</f>
         <v/>
       </c>
-      <c r="R13" s="52">
+      <c r="R13" s="51">
         <f>Расчёт!K13</f>
         <v/>
       </c>
-      <c r="S13" s="52">
+      <c r="S13" s="51">
         <f>IF(R13="","",RANK(R13,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -1973,13 +2048,13 @@
         </is>
       </c>
       <c r="C14" s="44" t="n">
-        <v>328.245041</v>
+        <v>331.544745</v>
       </c>
       <c r="D14" s="44" t="n">
-        <v>2794.774601</v>
+        <v>2822.869252</v>
       </c>
       <c r="E14" s="44" t="n">
-        <v>1052.269901</v>
+        <v>1052.427495</v>
       </c>
       <c r="F14" s="44" t="n">
         <v>351.735124</v>
@@ -1993,34 +2068,36 @@
       <c r="I14" s="45" t="n">
         <v>2.102234</v>
       </c>
-      <c r="J14" s="46" t="n"/>
-      <c r="K14" s="47" t="n"/>
-      <c r="L14" s="48" t="n"/>
-      <c r="M14" s="49">
+      <c r="J14" s="44" t="n">
+        <v>75</v>
+      </c>
+      <c r="K14" s="46" t="n"/>
+      <c r="L14" s="47" t="n"/>
+      <c r="M14" s="48">
         <f>IF(OR(E14="",F14="",F14=0),"",E14/F14-1)</f>
         <v/>
       </c>
-      <c r="N14" s="49">
+      <c r="N14" s="48">
         <f>IF(OR(G14="",H14="",H14=0),"",G14/H14-1)</f>
         <v/>
       </c>
-      <c r="O14" s="50">
+      <c r="O14" s="49">
         <f>IF(OR(C14="",E14="",E14=0),"",C14/E14)</f>
         <v/>
       </c>
-      <c r="P14" s="51">
+      <c r="P14" s="50">
         <f>IF(OR(C14="",I14="",I14=0),"",C14/I14)</f>
         <v/>
       </c>
-      <c r="Q14" s="50">
+      <c r="Q14" s="49">
         <f>IF(OR(C14="",D14="",C14=0),"",D14/C14)</f>
         <v/>
       </c>
-      <c r="R14" s="52">
+      <c r="R14" s="51">
         <f>Расчёт!K14</f>
         <v/>
       </c>
-      <c r="S14" s="52">
+      <c r="S14" s="51">
         <f>IF(R14="","",RANK(R14,$R$5:$R$14))</f>
         <v/>
       </c>
@@ -2047,7 +2124,7 @@
       <c r="S15" s="36" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="34">
-      <c r="A16" s="54" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>Легенда: зелёный — лучше среди сравниваемых, красный — хуже. Для Mcap/TVL, Mcap/Доход и FDV/Mcap меньше = лучше. Лидер по баллу подсвечен зелёным.</t>
         </is>
@@ -2072,7 +2149,7 @@
       <c r="S16" s="36" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="34">
-      <c r="A17" s="55" t="inlineStr">
+      <c r="A17" s="54" t="inlineStr">
         <is>
           <t>Балл относительный: показывает, кто сильнее внутри твоей выборки, а не «покупать/не покупать». Сравнивай сети одной категории.</t>
         </is>
@@ -2221,7 +2298,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="34">
-      <c r="A1" s="56" t="inlineStr">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Служебный лист: нормированные оценки 0–1 по каждой метрике</t>
         </is>
@@ -2320,66 +2397,66 @@
       <c r="AA3" s="36" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="34">
-      <c r="A4" s="56" t="inlineStr">
+      <c r="A4" s="55" t="inlineStr">
         <is>
           <t>Экосистема</t>
         </is>
       </c>
-      <c r="B4" s="56" t="inlineStr">
+      <c r="B4" s="55" t="inlineStr">
         <is>
           <t>Рост TVL 6м</t>
         </is>
       </c>
-      <c r="C4" s="56" t="inlineStr">
+      <c r="C4" s="55" t="inlineStr">
         <is>
           <t>Рост адресов 6м</t>
         </is>
       </c>
-      <c r="D4" s="56" t="inlineStr">
+      <c r="D4" s="55" t="inlineStr">
         <is>
           <t>Mcap / TVL</t>
         </is>
       </c>
-      <c r="E4" s="56" t="inlineStr">
+      <c r="E4" s="55" t="inlineStr">
         <is>
           <t>Mcap / Доход</t>
         </is>
       </c>
-      <c r="F4" s="56" t="inlineStr">
+      <c r="F4" s="55" t="inlineStr">
         <is>
           <t>Активных разработчиков</t>
         </is>
       </c>
-      <c r="G4" s="56" t="inlineStr">
+      <c r="G4" s="55" t="inlineStr">
         <is>
           <t>Разлок за 6 мес</t>
         </is>
       </c>
-      <c r="H4" s="56" t="inlineStr">
+      <c r="H4" s="55" t="inlineStr">
         <is>
           <t>FDV / Mcap</t>
         </is>
       </c>
-      <c r="I4" s="56" t="inlineStr">
+      <c r="I4" s="55" t="inlineStr">
         <is>
           <t>Инвесторы и команда</t>
         </is>
       </c>
-      <c r="J4" s="56" t="n"/>
-      <c r="K4" s="56" t="inlineStr">
+      <c r="J4" s="55" t="n"/>
+      <c r="K4" s="55" t="inlineStr">
         <is>
           <t>Итог 0–100</t>
         </is>
       </c>
-      <c r="L4" s="56" t="n"/>
-      <c r="M4" s="56" t="n"/>
-      <c r="N4" s="56" t="n"/>
-      <c r="O4" s="56" t="n"/>
-      <c r="P4" s="56" t="n"/>
-      <c r="Q4" s="56" t="n"/>
-      <c r="R4" s="56" t="n"/>
-      <c r="S4" s="56" t="n"/>
-      <c r="T4" s="56" t="n"/>
+      <c r="L4" s="55" t="n"/>
+      <c r="M4" s="55" t="n"/>
+      <c r="N4" s="55" t="n"/>
+      <c r="O4" s="55" t="n"/>
+      <c r="P4" s="55" t="n"/>
+      <c r="Q4" s="55" t="n"/>
+      <c r="R4" s="55" t="n"/>
+      <c r="S4" s="55" t="n"/>
+      <c r="T4" s="55" t="n"/>
       <c r="U4" s="36" t="n"/>
       <c r="V4" s="36" t="n"/>
       <c r="W4" s="36" t="n"/>
@@ -2393,40 +2470,40 @@
         <f>IF(Сравнение!A5="","",Сравнение!A5)</f>
         <v/>
       </c>
-      <c r="B5" s="57">
+      <c r="B5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M5)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M5-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C5" s="57">
+      <c r="C5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N5)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N5-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D5" s="57">
+      <c r="D5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O5)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O5)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E5" s="57">
+      <c r="E5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P5)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P5)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F5" s="57">
+      <c r="F5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J5)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J5-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G5" s="57">
+      <c r="G5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K5)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K5)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H5" s="57">
+      <c r="H5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q5)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q5)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I5" s="57">
+      <c r="I5" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L5)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L5-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J5" s="36" t="n"/>
-      <c r="K5" s="58">
+      <c r="K5" s="57">
         <f>IF(OR(Сравнение!A5="",SUM(T5:AA5)=0),"",100*SUM(L5:S5)/SUM(T5:AA5))</f>
         <v/>
       </c>
@@ -2500,40 +2577,40 @@
         <f>IF(Сравнение!A6="","",Сравнение!A6)</f>
         <v/>
       </c>
-      <c r="B6" s="57">
+      <c r="B6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M6)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M6-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C6" s="57">
+      <c r="C6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N6)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N6-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D6" s="57">
+      <c r="D6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O6)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O6)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E6" s="57">
+      <c r="E6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P6)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P6)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F6" s="57">
+      <c r="F6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J6)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J6-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G6" s="57">
+      <c r="G6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K6)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K6)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H6" s="57">
+      <c r="H6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q6)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q6)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I6" s="57">
+      <c r="I6" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L6)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L6-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J6" s="36" t="n"/>
-      <c r="K6" s="58">
+      <c r="K6" s="57">
         <f>IF(OR(Сравнение!A6="",SUM(T6:AA6)=0),"",100*SUM(L6:S6)/SUM(T6:AA6))</f>
         <v/>
       </c>
@@ -2607,40 +2684,40 @@
         <f>IF(Сравнение!A7="","",Сравнение!A7)</f>
         <v/>
       </c>
-      <c r="B7" s="57">
+      <c r="B7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M7)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M7-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C7" s="57">
+      <c r="C7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N7)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N7-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D7" s="57">
+      <c r="D7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O7)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O7)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E7" s="57">
+      <c r="E7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P7)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P7)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F7" s="57">
+      <c r="F7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J7)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J7-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G7" s="57">
+      <c r="G7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K7)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K7)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H7" s="57">
+      <c r="H7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q7)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q7)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I7" s="57">
+      <c r="I7" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L7)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L7-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J7" s="36" t="n"/>
-      <c r="K7" s="58">
+      <c r="K7" s="57">
         <f>IF(OR(Сравнение!A7="",SUM(T7:AA7)=0),"",100*SUM(L7:S7)/SUM(T7:AA7))</f>
         <v/>
       </c>
@@ -2714,40 +2791,40 @@
         <f>IF(Сравнение!A8="","",Сравнение!A8)</f>
         <v/>
       </c>
-      <c r="B8" s="57">
+      <c r="B8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M8)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M8-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C8" s="57">
+      <c r="C8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N8)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N8-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D8" s="57">
+      <c r="D8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O8)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O8)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E8" s="57">
+      <c r="E8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P8)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P8)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F8" s="57">
+      <c r="F8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J8)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J8-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G8" s="57">
+      <c r="G8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K8)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K8)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H8" s="57">
+      <c r="H8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q8)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q8)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I8" s="57">
+      <c r="I8" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L8)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L8-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J8" s="36" t="n"/>
-      <c r="K8" s="58">
+      <c r="K8" s="57">
         <f>IF(OR(Сравнение!A8="",SUM(T8:AA8)=0),"",100*SUM(L8:S8)/SUM(T8:AA8))</f>
         <v/>
       </c>
@@ -2821,40 +2898,40 @@
         <f>IF(Сравнение!A9="","",Сравнение!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="57">
+      <c r="B9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M9)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M9-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C9" s="57">
+      <c r="C9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N9)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N9-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D9" s="57">
+      <c r="D9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O9)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O9)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E9" s="57">
+      <c r="E9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P9)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P9)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F9" s="57">
+      <c r="F9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J9)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J9-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G9" s="57">
+      <c r="G9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K9)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K9)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H9" s="57">
+      <c r="H9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q9)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q9)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I9" s="57">
+      <c r="I9" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L9)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L9-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J9" s="36" t="n"/>
-      <c r="K9" s="58">
+      <c r="K9" s="57">
         <f>IF(OR(Сравнение!A9="",SUM(T9:AA9)=0),"",100*SUM(L9:S9)/SUM(T9:AA9))</f>
         <v/>
       </c>
@@ -2928,40 +3005,40 @@
         <f>IF(Сравнение!A10="","",Сравнение!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="57">
+      <c r="B10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M10)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M10-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C10" s="57">
+      <c r="C10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N10)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N10-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D10" s="57">
+      <c r="D10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O10)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O10)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E10" s="57">
+      <c r="E10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P10)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P10)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F10" s="57">
+      <c r="F10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J10)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J10-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G10" s="57">
+      <c r="G10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K10)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K10)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H10" s="57">
+      <c r="H10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q10)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q10)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I10" s="57">
+      <c r="I10" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L10)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L10-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J10" s="36" t="n"/>
-      <c r="K10" s="58">
+      <c r="K10" s="57">
         <f>IF(OR(Сравнение!A10="",SUM(T10:AA10)=0),"",100*SUM(L10:S10)/SUM(T10:AA10))</f>
         <v/>
       </c>
@@ -3035,40 +3112,40 @@
         <f>IF(Сравнение!A11="","",Сравнение!A11)</f>
         <v/>
       </c>
-      <c r="B11" s="57">
+      <c r="B11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M11)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M11-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C11" s="57">
+      <c r="C11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N11)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N11-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D11" s="57">
+      <c r="D11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O11)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O11)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E11" s="57">
+      <c r="E11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P11)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P11)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F11" s="57">
+      <c r="F11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J11)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J11-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G11" s="57">
+      <c r="G11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K11)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K11)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H11" s="57">
+      <c r="H11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q11)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q11)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I11" s="57">
+      <c r="I11" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L11)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L11-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J11" s="36" t="n"/>
-      <c r="K11" s="58">
+      <c r="K11" s="57">
         <f>IF(OR(Сравнение!A11="",SUM(T11:AA11)=0),"",100*SUM(L11:S11)/SUM(T11:AA11))</f>
         <v/>
       </c>
@@ -3142,40 +3219,40 @@
         <f>IF(Сравнение!A12="","",Сравнение!A12)</f>
         <v/>
       </c>
-      <c r="B12" s="57">
+      <c r="B12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M12)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M12-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C12" s="57">
+      <c r="C12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N12)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N12-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D12" s="57">
+      <c r="D12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O12)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O12)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E12" s="57">
+      <c r="E12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P12)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P12)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F12" s="57">
+      <c r="F12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J12)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J12-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G12" s="57">
+      <c r="G12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K12)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K12)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H12" s="57">
+      <c r="H12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q12)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q12)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I12" s="57">
+      <c r="I12" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L12)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L12-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J12" s="36" t="n"/>
-      <c r="K12" s="58">
+      <c r="K12" s="57">
         <f>IF(OR(Сравнение!A12="",SUM(T12:AA12)=0),"",100*SUM(L12:S12)/SUM(T12:AA12))</f>
         <v/>
       </c>
@@ -3249,40 +3326,40 @@
         <f>IF(Сравнение!A13="","",Сравнение!A13)</f>
         <v/>
       </c>
-      <c r="B13" s="57">
+      <c r="B13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M13)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M13-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C13" s="57">
+      <c r="C13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N13)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N13-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O13)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O13)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E13" s="57">
+      <c r="E13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P13)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P13)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F13" s="57">
+      <c r="F13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J13)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J13-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G13" s="57">
+      <c r="G13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K13)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K13)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H13" s="57">
+      <c r="H13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q13)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q13)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I13" s="57">
+      <c r="I13" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L13)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L13-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J13" s="36" t="n"/>
-      <c r="K13" s="58">
+      <c r="K13" s="57">
         <f>IF(OR(Сравнение!A13="",SUM(T13:AA13)=0),"",100*SUM(L13:S13)/SUM(T13:AA13))</f>
         <v/>
       </c>
@@ -3356,40 +3433,40 @@
         <f>IF(Сравнение!A14="","",Сравнение!A14)</f>
         <v/>
       </c>
-      <c r="B14" s="57">
+      <c r="B14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!M14)),COUNT(Сравнение!$M$5:$M$14)&lt;2),"",IF(MAX(Сравнение!$M$5:$M$14)=MIN(Сравнение!$M$5:$M$14),0.5,(Сравнение!M14-MIN(Сравнение!$M$5:$M$14))/(MAX(Сравнение!$M$5:$M$14)-MIN(Сравнение!$M$5:$M$14))))</f>
         <v/>
       </c>
-      <c r="C14" s="57">
+      <c r="C14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!N14)),COUNT(Сравнение!$N$5:$N$14)&lt;2),"",IF(MAX(Сравнение!$N$5:$N$14)=MIN(Сравнение!$N$5:$N$14),0.5,(Сравнение!N14-MIN(Сравнение!$N$5:$N$14))/(MAX(Сравнение!$N$5:$N$14)-MIN(Сравнение!$N$5:$N$14))))</f>
         <v/>
       </c>
-      <c r="D14" s="57">
+      <c r="D14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!O14)),COUNT(Сравнение!$O$5:$O$14)&lt;2),"",IF(MAX(Сравнение!$O$5:$O$14)=MIN(Сравнение!$O$5:$O$14),0.5,(MAX(Сравнение!$O$5:$O$14)-Сравнение!O14)/(MAX(Сравнение!$O$5:$O$14)-MIN(Сравнение!$O$5:$O$14))))</f>
         <v/>
       </c>
-      <c r="E14" s="57">
+      <c r="E14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!P14)),COUNT(Сравнение!$P$5:$P$14)&lt;2),"",IF(MAX(Сравнение!$P$5:$P$14)=MIN(Сравнение!$P$5:$P$14),0.5,(MAX(Сравнение!$P$5:$P$14)-Сравнение!P14)/(MAX(Сравнение!$P$5:$P$14)-MIN(Сравнение!$P$5:$P$14))))</f>
         <v/>
       </c>
-      <c r="F14" s="57">
+      <c r="F14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!J14)),COUNT(Сравнение!$J$5:$J$14)&lt;2),"",IF(MAX(Сравнение!$J$5:$J$14)=MIN(Сравнение!$J$5:$J$14),0.5,(Сравнение!J14-MIN(Сравнение!$J$5:$J$14))/(MAX(Сравнение!$J$5:$J$14)-MIN(Сравнение!$J$5:$J$14))))</f>
         <v/>
       </c>
-      <c r="G14" s="57">
+      <c r="G14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!K14)),COUNT(Сравнение!$K$5:$K$14)&lt;2),"",IF(MAX(Сравнение!$K$5:$K$14)=MIN(Сравнение!$K$5:$K$14),0.5,(MAX(Сравнение!$K$5:$K$14)-Сравнение!K14)/(MAX(Сравнение!$K$5:$K$14)-MIN(Сравнение!$K$5:$K$14))))</f>
         <v/>
       </c>
-      <c r="H14" s="57">
+      <c r="H14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!Q14)),COUNT(Сравнение!$Q$5:$Q$14)&lt;2),"",IF(MAX(Сравнение!$Q$5:$Q$14)=MIN(Сравнение!$Q$5:$Q$14),0.5,(MAX(Сравнение!$Q$5:$Q$14)-Сравнение!Q14)/(MAX(Сравнение!$Q$5:$Q$14)-MIN(Сравнение!$Q$5:$Q$14))))</f>
         <v/>
       </c>
-      <c r="I14" s="57">
+      <c r="I14" s="56">
         <f>IF(OR(NOT(ISNUMBER(Сравнение!L14)),COUNT(Сравнение!$L$5:$L$14)&lt;2),"",IF(MAX(Сравнение!$L$5:$L$14)=MIN(Сравнение!$L$5:$L$14),0.5,(Сравнение!L14-MIN(Сравнение!$L$5:$L$14))/(MAX(Сравнение!$L$5:$L$14)-MIN(Сравнение!$L$5:$L$14))))</f>
         <v/>
       </c>
       <c r="J14" s="36" t="n"/>
-      <c r="K14" s="58">
+      <c r="K14" s="57">
         <f>IF(OR(Сравнение!A14="",SUM(T14:AA14)=0),"",100*SUM(L14:S14)/SUM(T14:AA14))</f>
         <v/>
       </c>
@@ -3480,7 +3557,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="34">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Веса метрик (меняй под себя)</t>
         </is>
@@ -3494,149 +3571,149 @@
       <c r="C2" s="36" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1" s="34">
-      <c r="A3" s="60" t="inlineStr">
+      <c r="A3" s="59" t="inlineStr">
         <is>
           <t>Метрика</t>
         </is>
       </c>
-      <c r="B3" s="60" t="inlineStr">
+      <c r="B3" s="59" t="inlineStr">
         <is>
           <t>Вес</t>
         </is>
       </c>
-      <c r="C3" s="60" t="inlineStr">
+      <c r="C3" s="59" t="inlineStr">
         <is>
           <t>Направление</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="34">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>Рост TVL 6м</t>
         </is>
       </c>
-      <c r="B4" s="62" t="n">
+      <c r="B4" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="C4" s="63" t="inlineStr">
+      <c r="C4" s="62" t="inlineStr">
         <is>
           <t>больше = лучше</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="34">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>Рост адресов 6м</t>
         </is>
       </c>
-      <c r="B5" s="62" t="n">
+      <c r="B5" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="63" t="inlineStr">
+      <c r="C5" s="62" t="inlineStr">
         <is>
           <t>больше = лучше</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="34">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>Mcap / TVL</t>
         </is>
       </c>
-      <c r="B6" s="62" t="n">
+      <c r="B6" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="63" t="inlineStr">
+      <c r="C6" s="62" t="inlineStr">
         <is>
           <t>меньше = лучше</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="34">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>Mcap / Доход</t>
         </is>
       </c>
-      <c r="B7" s="62" t="n">
+      <c r="B7" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="C7" s="63" t="inlineStr">
+      <c r="C7" s="62" t="inlineStr">
         <is>
           <t>меньше = лучше</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="34">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>Активных разработчиков</t>
         </is>
       </c>
-      <c r="B8" s="62" t="n">
+      <c r="B8" s="61" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="63" t="inlineStr">
+      <c r="C8" s="62" t="inlineStr">
         <is>
           <t>больше = лучше</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="34">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>Разлок за 6 мес</t>
         </is>
       </c>
-      <c r="B9" s="62" t="n">
+      <c r="B9" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="C9" s="63" t="inlineStr">
+      <c r="C9" s="62" t="inlineStr">
         <is>
           <t>меньше = лучше</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="34">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>FDV / Mcap</t>
         </is>
       </c>
-      <c r="B10" s="62" t="n">
+      <c r="B10" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="63" t="inlineStr">
+      <c r="C10" s="62" t="inlineStr">
         <is>
           <t>меньше = лучше</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="34">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>Инвесторы и команда</t>
         </is>
       </c>
-      <c r="B11" s="62" t="n">
+      <c r="B11" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="63" t="inlineStr">
+      <c r="C11" s="62" t="inlineStr">
         <is>
           <t>больше = лучше</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="34">
-      <c r="A12" s="56" t="inlineStr">
+      <c r="A12" s="55" t="inlineStr">
         <is>
           <t>Сумма весов</t>
         </is>
       </c>
-      <c r="B12" s="56">
+      <c r="B12" s="55">
         <f>SUM(B4:B11)</f>
         <v/>
       </c>
@@ -3664,260 +3741,260 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="34">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Где брать цифры</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="34">
-      <c r="A3" s="64" t="inlineStr">
+      <c r="A3" s="63" t="inlineStr">
         <is>
           <t>Колонка</t>
         </is>
       </c>
-      <c r="B3" s="64" t="inlineStr">
+      <c r="B3" s="63" t="inlineStr">
         <is>
           <t>Источник</t>
         </is>
       </c>
-      <c r="C3" s="64" t="inlineStr">
+      <c r="C3" s="63" t="inlineStr">
         <is>
           <t>Ссылка</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="34">
-      <c r="A4" s="65" t="inlineStr">
+      <c r="A4" s="64" t="inlineStr">
         <is>
           <t>Капитализация, FDV</t>
         </is>
       </c>
-      <c r="B4" s="65" t="inlineStr">
+      <c r="B4" s="64" t="inlineStr">
         <is>
           <t>CoinGecko</t>
         </is>
       </c>
-      <c r="C4" s="66" t="inlineStr">
+      <c r="C4" s="65" t="inlineStr">
         <is>
           <t>https://www.coingecko.com/en/categories</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="34">
-      <c r="A5" s="65" t="inlineStr">
+      <c r="A5" s="64" t="inlineStr">
         <is>
           <t>TVL сейчас и 6 мес назад</t>
         </is>
       </c>
-      <c r="B5" s="65" t="inlineStr">
+      <c r="B5" s="64" t="inlineStr">
         <is>
           <t>DeFiLlama → Chains</t>
         </is>
       </c>
-      <c r="C5" s="66" t="inlineStr">
+      <c r="C5" s="65" t="inlineStr">
         <is>
           <t>https://defillama.com/chains</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="34">
-      <c r="A6" s="65" t="inlineStr">
+      <c r="A6" s="64" t="inlineStr">
         <is>
           <t>Активные адреса</t>
         </is>
       </c>
-      <c r="B6" s="65" t="inlineStr">
+      <c r="B6" s="64" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="C6" s="66" t="inlineStr">
+      <c r="C6" s="65" t="inlineStr">
         <is>
           <t>https://app.artemis.xyz</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="34">
-      <c r="A7" s="65" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>Доход / комиссии</t>
         </is>
       </c>
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>DeFiLlama Fees</t>
         </is>
       </c>
-      <c r="C7" s="66" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>https://defillama.com/fees</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="34">
-      <c r="A8" s="65" t="inlineStr">
+      <c r="A8" s="64" t="inlineStr">
         <is>
           <t>Доход (альтернатива)</t>
         </is>
       </c>
-      <c r="B8" s="65" t="inlineStr">
+      <c r="B8" s="64" t="inlineStr">
         <is>
           <t>Token Terminal</t>
         </is>
       </c>
-      <c r="C8" s="66" t="inlineStr">
+      <c r="C8" s="65" t="inlineStr">
         <is>
           <t>https://tokenterminal.com</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="34">
-      <c r="A9" s="65" t="inlineStr">
+      <c r="A9" s="64" t="inlineStr">
         <is>
           <t>Разработчики</t>
         </is>
       </c>
-      <c r="B9" s="65" t="inlineStr">
+      <c r="B9" s="64" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="C9" s="66" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>https://app.artemis.xyz</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="34">
-      <c r="A10" s="65" t="inlineStr">
+      <c r="A10" s="64" t="inlineStr">
         <is>
           <t>Разлоки</t>
         </is>
       </c>
-      <c r="B10" s="65" t="inlineStr">
+      <c r="B10" s="64" t="inlineStr">
         <is>
           <t>Tokenomist</t>
         </is>
       </c>
-      <c r="C10" s="66" t="inlineStr">
+      <c r="C10" s="65" t="inlineStr">
         <is>
           <t>https://tokenomist.ai</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="34">
-      <c r="A11" s="65" t="inlineStr">
+      <c r="A11" s="64" t="inlineStr">
         <is>
           <t>Инвесторы, раунды</t>
         </is>
       </c>
-      <c r="B11" s="65" t="inlineStr">
+      <c r="B11" s="64" t="inlineStr">
         <is>
           <t>CryptoRank</t>
         </is>
       </c>
-      <c r="C11" s="66" t="inlineStr">
+      <c r="C11" s="65" t="inlineStr">
         <is>
           <t>https://cryptorank.io</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="34">
-      <c r="A12" s="65" t="inlineStr">
+      <c r="A12" s="64" t="inlineStr">
         <is>
           <t>Инвесторы, раунды</t>
         </is>
       </c>
-      <c r="B12" s="65" t="inlineStr">
+      <c r="B12" s="64" t="inlineStr">
         <is>
           <t>DeFiLlama Raises</t>
         </is>
       </c>
-      <c r="C12" s="66" t="inlineStr">
+      <c r="C12" s="65" t="inlineStr">
         <is>
           <t>https://defillama.com/raises</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="34">
-      <c r="A13" s="65" t="inlineStr">
+      <c r="A13" s="64" t="inlineStr">
         <is>
           <t>Метрики L2</t>
         </is>
       </c>
-      <c r="B13" s="65" t="inlineStr">
+      <c r="B13" s="64" t="inlineStr">
         <is>
           <t>growthepie</t>
         </is>
       </c>
-      <c r="C13" s="66" t="inlineStr">
+      <c r="C13" s="65" t="inlineStr">
         <is>
           <t>https://www.growthepie.xyz</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="34">
-      <c r="A14" s="65" t="inlineStr">
+      <c r="A14" s="64" t="inlineStr">
         <is>
           <t>Риски L2</t>
         </is>
       </c>
-      <c r="B14" s="65" t="inlineStr">
+      <c r="B14" s="64" t="inlineStr">
         <is>
           <t>L2BEAT</t>
         </is>
       </c>
-      <c r="C14" s="66" t="inlineStr">
+      <c r="C14" s="65" t="inlineStr">
         <is>
           <t>https://l2beat.com</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="34">
-      <c r="A17" s="67" t="inlineStr">
+      <c r="A17" s="66" t="inlineStr">
         <is>
           <t>Как пользоваться:</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="34">
-      <c r="A18" s="68" t="inlineStr">
+      <c r="A18" s="67" t="inlineStr">
         <is>
           <t>1. На листе «Сравнение» замени строки «Пример» своими сетями (до 10 штук).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="34">
-      <c r="A19" s="68" t="inlineStr">
+      <c r="A19" s="67" t="inlineStr">
         <is>
           <t>2. Заполняй жёлтые ячейки. Пустые метрики просто не учитываются в балле.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="34">
-      <c r="A20" s="68" t="inlineStr">
+      <c r="A20" s="67" t="inlineStr">
         <is>
           <t>3. Для балла нужно минимум 2 сети с данными по метрике.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="34">
-      <c r="A21" s="68" t="inlineStr">
+      <c r="A21" s="67" t="inlineStr">
         <is>
           <t>4. Веса метрик меняй на листе «Веса».</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="34">
-      <c r="A22" s="68" t="inlineStr">
+      <c r="A22" s="67" t="inlineStr">
         <is>
           <t>5. Разлок вводи в процентах (3% = 3%), инвесторов — оценкой 1–5 по своему мнению.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="34">
-      <c r="A23" s="68" t="inlineStr">
+      <c r="A23" s="67" t="inlineStr">
         <is>
           <t>Балл относительный и не является рекомендацией к покупке.</t>
         </is>
@@ -3960,34 +4037,34 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>Откуда взята каждая цифра (сбор 30.09.2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="70" t="inlineStr">
+      <c r="A3" s="69" t="inlineStr">
         <is>
           <t>Экосистема</t>
         </is>
       </c>
-      <c r="B3" s="70" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
           <t>Метрика</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="69" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="D3" s="70" t="inlineStr">
+      <c r="D3" s="69" t="inlineStr">
         <is>
           <t>Источник</t>
         </is>
       </c>
-      <c r="E3" s="70" t="inlineStr">
+      <c r="E3" s="69" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -4004,8 +4081,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C4" s="71" t="n">
-        <v>327258.690254</v>
+      <c r="C4" s="70" t="n">
+        <v>327944.680337</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -4025,8 +4102,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C5" s="71" t="n">
-        <v>327258.690254</v>
+      <c r="C5" s="70" t="n">
+        <v>327944.680337</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -4046,8 +4123,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C6" s="71" t="n">
-        <v>53918.369868</v>
+      <c r="C6" s="70" t="n">
+        <v>53303.04256</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -4071,7 +4148,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C7" s="71" t="n">
+      <c r="C7" s="70" t="n">
         <v>53909.531522</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -4096,7 +4173,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C8" s="71" t="n">
+      <c r="C8" s="70" t="n">
         <v>495105</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -4121,7 +4198,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C9" s="71" t="n">
+      <c r="C9" s="70" t="n">
         <v>616284</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -4146,7 +4223,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C10" s="71" t="n">
+      <c r="C10" s="70" t="n">
         <v>202.689948</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -4161,61 +4238,67 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="72" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="B11" s="72" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C11" s="73" t="n"/>
-      <c r="D11" s="72" t="inlineStr">
+      <c r="C11" s="70" t="n">
+        <v>3270</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="71" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B12" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C12" s="72" t="n"/>
+      <c r="D12" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E11" s="72" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="72" t="inlineStr">
+      <c r="E12" s="71" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="71" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="B12" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C12" s="74" t="n"/>
-      <c r="D12" s="72" t="inlineStr">
+      <c r="B13" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C13" s="73" t="n"/>
+      <c r="D13" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E12" s="72" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="72" t="inlineStr">
-        <is>
-          <t>Ethereum</t>
-        </is>
-      </c>
-      <c r="B13" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C13" s="73" t="n"/>
-      <c r="D13" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E13" s="72" t="inlineStr"/>
+      <c r="E13" s="71" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4228,8 +4311,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C14" s="71" t="n">
-        <v>69988.26169699999</v>
+      <c r="C14" s="70" t="n">
+        <v>70355.204557</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -4249,8 +4332,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C15" s="71" t="n">
-        <v>75581.369252</v>
+      <c r="C15" s="70" t="n">
+        <v>75977.633946</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -4270,8 +4353,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C16" s="71" t="n">
-        <v>6471.36886</v>
+      <c r="C16" s="70" t="n">
+        <v>6568.178533</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4295,7 +4378,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C17" s="71" t="n">
+      <c r="C17" s="70" t="n">
         <v>6357.767767</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -4320,7 +4403,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C18" s="71" t="n">
+      <c r="C18" s="70" t="n">
         <v>5123259</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -4345,7 +4428,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C19" s="71" t="n">
+      <c r="C19" s="70" t="n">
         <v>4289374</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -4370,7 +4453,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C20" s="71" t="n">
+      <c r="C20" s="70" t="n">
         <v>239.426752</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -4385,61 +4468,67 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="72" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Solana</t>
         </is>
       </c>
-      <c r="B21" s="72" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C21" s="73" t="n"/>
-      <c r="D21" s="72" t="inlineStr">
+      <c r="C21" s="70" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="71" t="inlineStr">
+        <is>
+          <t>Solana</t>
+        </is>
+      </c>
+      <c r="B22" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C22" s="72" t="n"/>
+      <c r="D22" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E21" s="72" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="72" t="inlineStr">
+      <c r="E22" s="71" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="71" t="inlineStr">
         <is>
           <t>Solana</t>
         </is>
       </c>
-      <c r="B22" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C22" s="74" t="n"/>
-      <c r="D22" s="72" t="inlineStr">
+      <c r="B23" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C23" s="73" t="n"/>
+      <c r="D23" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E22" s="72" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="72" t="inlineStr">
-        <is>
-          <t>Solana</t>
-        </is>
-      </c>
-      <c r="B23" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C23" s="73" t="n"/>
-      <c r="D23" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E23" s="72" t="inlineStr"/>
+      <c r="E23" s="71" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4452,8 +4541,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C24" s="71" t="n">
-        <v>4767.521283</v>
+      <c r="C24" s="70" t="n">
+        <v>4865.721245</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -4473,8 +4562,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C25" s="71" t="n">
-        <v>11637.930067</v>
+      <c r="C25" s="70" t="n">
+        <v>11877.644633</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -4494,8 +4583,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C26" s="71" t="n">
-        <v>559.329125</v>
+      <c r="C26" s="70" t="n">
+        <v>551.750347</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -4519,7 +4608,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C27" s="71" t="n">
+      <c r="C27" s="70" t="n">
         <v>570.720387</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -4544,7 +4633,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C28" s="71" t="n">
+      <c r="C28" s="70" t="n">
         <v>134536</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -4569,7 +4658,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C29" s="71" t="n">
+      <c r="C29" s="70" t="n">
         <v>229146</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -4594,7 +4683,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C30" s="71" t="n">
+      <c r="C30" s="70" t="n">
         <v>3.512066</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -4609,61 +4698,67 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="72" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Sui</t>
         </is>
       </c>
-      <c r="B31" s="72" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C31" s="73" t="n"/>
-      <c r="D31" s="72" t="inlineStr">
+      <c r="C31" s="70" t="n">
+        <v>254</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="71" t="inlineStr">
+        <is>
+          <t>Sui</t>
+        </is>
+      </c>
+      <c r="B32" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E31" s="72" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="72" t="inlineStr">
+      <c r="E32" s="71" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="71" t="inlineStr">
         <is>
           <t>Sui</t>
         </is>
       </c>
-      <c r="B32" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C32" s="74" t="n"/>
-      <c r="D32" s="72" t="inlineStr">
+      <c r="B33" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C33" s="73" t="n"/>
+      <c r="D33" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E32" s="72" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="72" t="inlineStr">
-        <is>
-          <t>Sui</t>
-        </is>
-      </c>
-      <c r="B33" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C33" s="73" t="n"/>
-      <c r="D33" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E33" s="72" t="inlineStr"/>
+      <c r="E33" s="71" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4676,8 +4771,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C34" s="71" t="n">
-        <v>687.9191049999999</v>
+      <c r="C34" s="70" t="n">
+        <v>690.49137</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -4697,8 +4792,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C35" s="71" t="n">
-        <v>955.210046</v>
+      <c r="C35" s="70" t="n">
+        <v>958.7853270000001</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -4718,8 +4813,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C36" s="71" t="n">
-        <v>55.740282</v>
+      <c r="C36" s="70" t="n">
+        <v>55.53995</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -4743,7 +4838,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C37" s="71" t="n">
+      <c r="C37" s="70" t="n">
         <v>285.748159</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -4758,25 +4853,25 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="75" t="inlineStr">
+      <c r="A38" s="74" t="inlineStr">
         <is>
           <t>Aptos</t>
         </is>
       </c>
-      <c r="B38" s="75" t="inlineStr">
+      <c r="B38" s="74" t="inlineStr">
         <is>
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C38" s="76" t="n">
+      <c r="C38" s="75" t="n">
         <v>35921</v>
       </c>
-      <c r="D38" s="75" t="inlineStr">
+      <c r="D38" s="74" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="E38" s="75" t="inlineStr">
+      <c r="E38" s="74" t="inlineStr">
         <is>
           <t>медиана за 7 дн до 2026-09-29. ⚠ изменение за 6 мес больше чем в 10 раз — проверь, реально ли это</t>
         </is>
@@ -4793,7 +4888,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C39" s="71" t="n">
+      <c r="C39" s="70" t="n">
         <v>1055333</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -4818,7 +4913,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C40" s="71" t="n">
+      <c r="C40" s="70" t="n">
         <v>1.145126</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -4833,61 +4928,67 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="72" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Aptos</t>
         </is>
       </c>
-      <c r="B41" s="72" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C41" s="73" t="n"/>
-      <c r="D41" s="72" t="inlineStr">
+      <c r="C41" s="70" t="n">
+        <v>92</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="71" t="inlineStr">
+        <is>
+          <t>Aptos</t>
+        </is>
+      </c>
+      <c r="B42" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C42" s="72" t="n"/>
+      <c r="D42" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E41" s="72" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="72" t="inlineStr">
+      <c r="E42" s="71" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="71" t="inlineStr">
         <is>
           <t>Aptos</t>
         </is>
       </c>
-      <c r="B42" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C42" s="74" t="n"/>
-      <c r="D42" s="72" t="inlineStr">
+      <c r="B43" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C43" s="73" t="n"/>
+      <c r="D43" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E42" s="72" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="72" t="inlineStr">
-        <is>
-          <t>Aptos</t>
-        </is>
-      </c>
-      <c r="B43" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C43" s="73" t="n"/>
-      <c r="D43" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E43" s="72" t="inlineStr"/>
+      <c r="E43" s="71" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4900,8 +5001,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C44" s="71" t="n">
-        <v>4829.34046</v>
+      <c r="C44" s="70" t="n">
+        <v>4879.641119</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -4921,8 +5022,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C45" s="71" t="n">
-        <v>5120.001442</v>
+      <c r="C45" s="70" t="n">
+        <v>5173.313795</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -4942,8 +5043,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C46" s="71" t="n">
-        <v>640.767554</v>
+      <c r="C46" s="70" t="n">
+        <v>626.279733</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -4967,7 +5068,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C47" s="71" t="n">
+      <c r="C47" s="70" t="n">
         <v>724.301796</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -4982,50 +5083,50 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="75" t="inlineStr">
+      <c r="A48" s="74" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>
       </c>
-      <c r="B48" s="75" t="inlineStr">
+      <c r="B48" s="74" t="inlineStr">
         <is>
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C48" s="76" t="n">
+      <c r="C48" s="75" t="n">
         <v>21091</v>
       </c>
-      <c r="D48" s="75" t="inlineStr">
+      <c r="D48" s="74" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="E48" s="75" t="inlineStr">
+      <c r="E48" s="74" t="inlineStr">
         <is>
           <t>медиана за 7 дн до 2026-09-29. ⚠ ступенька в данных около 2026-07-11: медиана 502,037 → 22,052 за неделю — возможна смена методики источника, проверь вручную</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="75" t="inlineStr">
+      <c r="A49" s="74" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>
       </c>
-      <c r="B49" s="75" t="inlineStr">
+      <c r="B49" s="74" t="inlineStr">
         <is>
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C49" s="76" t="n">
+      <c r="C49" s="75" t="n">
         <v>643627</v>
       </c>
-      <c r="D49" s="75" t="inlineStr">
+      <c r="D49" s="74" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="E49" s="75" t="inlineStr">
+      <c r="E49" s="74" t="inlineStr">
         <is>
           <t>медиана за 7 дн до 2026-04-01. ⚠ ступенька в данных около 2026-07-11: медиана 502,037 → 22,052 за неделю — возможна смена методики источника, проверь вручную</t>
         </is>
@@ -5042,7 +5143,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C50" s="71" t="n">
+      <c r="C50" s="70" t="n">
         <v>4.076565</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -5057,61 +5158,67 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="72" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>
       </c>
-      <c r="B51" s="72" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C51" s="73" t="n"/>
-      <c r="D51" s="72" t="inlineStr">
+      <c r="C51" s="70" t="n">
+        <v>108</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="71" t="inlineStr">
+        <is>
+          <t>Avalanche</t>
+        </is>
+      </c>
+      <c r="B52" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C52" s="72" t="n"/>
+      <c r="D52" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E51" s="72" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="72" t="inlineStr">
+      <c r="E52" s="71" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="71" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>
       </c>
-      <c r="B52" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C52" s="74" t="n"/>
-      <c r="D52" s="72" t="inlineStr">
+      <c r="B53" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C53" s="73" t="n"/>
+      <c r="D53" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E52" s="72" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="72" t="inlineStr">
-        <is>
-          <t>Avalanche</t>
-        </is>
-      </c>
-      <c r="B53" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C53" s="73" t="n"/>
-      <c r="D53" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E53" s="72" t="inlineStr"/>
+      <c r="E53" s="71" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5124,8 +5231,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C54" s="71" t="n">
-        <v>6908.777867</v>
+      <c r="C54" s="70" t="n">
+        <v>7048.836656</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -5145,8 +5252,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C55" s="71" t="n">
-        <v>6908.778987</v>
+      <c r="C55" s="70" t="n">
+        <v>7048.837611</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -5166,8 +5273,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C56" s="71" t="n">
-        <v>239.929727</v>
+      <c r="C56" s="70" t="n">
+        <v>236.616937</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -5191,7 +5298,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C57" s="71" t="n">
+      <c r="C57" s="70" t="n">
         <v>95.21909100000001</v>
       </c>
       <c r="D57" t="inlineStr">
@@ -5206,50 +5313,50 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="75" t="inlineStr">
+      <c r="A58" s="74" t="inlineStr">
         <is>
           <t>Near</t>
         </is>
       </c>
-      <c r="B58" s="75" t="inlineStr">
+      <c r="B58" s="74" t="inlineStr">
         <is>
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C58" s="76" t="n">
+      <c r="C58" s="75" t="n">
         <v>76790</v>
       </c>
-      <c r="D58" s="75" t="inlineStr">
+      <c r="D58" s="74" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="E58" s="75" t="inlineStr">
+      <c r="E58" s="74" t="inlineStr">
         <is>
           <t>медиана за 7 дн до 2026-09-29. ⚠ ступенька в данных около 2026-03-30: медиана 3,067,142 → 472,650 за неделю — возможна смена методики источника, проверь вручную</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="75" t="inlineStr">
+      <c r="A59" s="74" t="inlineStr">
         <is>
           <t>Near</t>
         </is>
       </c>
-      <c r="B59" s="75" t="inlineStr">
+      <c r="B59" s="74" t="inlineStr">
         <is>
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C59" s="76" t="n">
+      <c r="C59" s="75" t="n">
         <v>3067142</v>
       </c>
-      <c r="D59" s="75" t="inlineStr">
+      <c r="D59" s="74" t="inlineStr">
         <is>
           <t>Artemis</t>
         </is>
       </c>
-      <c r="E59" s="75" t="inlineStr">
+      <c r="E59" s="74" t="inlineStr">
         <is>
           <t>медиана за 7 дн до 2026-04-01. ⚠ ступенька в данных около 2026-03-30: медиана 3,067,142 → 472,650 за неделю — возможна смена методики источника, проверь вручную</t>
         </is>
@@ -5266,7 +5373,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C60" s="71" t="n">
+      <c r="C60" s="70" t="n">
         <v>1.261909</v>
       </c>
       <c r="D60" t="inlineStr">
@@ -5281,61 +5388,67 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="72" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Near</t>
         </is>
       </c>
-      <c r="B61" s="72" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C61" s="73" t="n"/>
-      <c r="D61" s="72" t="inlineStr">
+      <c r="C61" s="70" t="n">
+        <v>150</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="71" t="inlineStr">
+        <is>
+          <t>Near</t>
+        </is>
+      </c>
+      <c r="B62" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C62" s="72" t="n"/>
+      <c r="D62" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E61" s="72" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="72" t="inlineStr">
+      <c r="E62" s="71" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="71" t="inlineStr">
         <is>
           <t>Near</t>
         </is>
       </c>
-      <c r="B62" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C62" s="74" t="n"/>
-      <c r="D62" s="72" t="inlineStr">
+      <c r="B63" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C63" s="73" t="n"/>
+      <c r="D63" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E62" s="72" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="72" t="inlineStr">
-        <is>
-          <t>Near</t>
-        </is>
-      </c>
-      <c r="B63" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C63" s="73" t="n"/>
-      <c r="D63" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E63" s="72" t="inlineStr"/>
+      <c r="E63" s="71" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5348,8 +5461,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C64" s="71" t="n">
-        <v>4228.799095</v>
+      <c r="C64" s="70" t="n">
+        <v>4238.049641</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -5369,8 +5482,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C65" s="71" t="n">
-        <v>7895.284465</v>
+      <c r="C65" s="70" t="n">
+        <v>7912.528129</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -5390,8 +5503,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C66" s="71" t="n">
-        <v>55.149255</v>
+      <c r="C66" s="70" t="n">
+        <v>54.352401</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -5415,7 +5528,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C67" s="71" t="n">
+      <c r="C67" s="70" t="n">
         <v>55.174661</v>
       </c>
       <c r="D67" t="inlineStr">
@@ -5440,7 +5553,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C68" s="71" t="n">
+      <c r="C68" s="70" t="n">
         <v>103801</v>
       </c>
       <c r="D68" t="inlineStr">
@@ -5465,7 +5578,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C69" s="71" t="n">
+      <c r="C69" s="70" t="n">
         <v>69929</v>
       </c>
       <c r="D69" t="inlineStr">
@@ -5490,7 +5603,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C70" s="71" t="n">
+      <c r="C70" s="70" t="n">
         <v>2.119862</v>
       </c>
       <c r="D70" t="inlineStr">
@@ -5505,61 +5618,67 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="72" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>TON</t>
         </is>
       </c>
-      <c r="B71" s="72" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C71" s="73" t="n"/>
-      <c r="D71" s="72" t="inlineStr">
+      <c r="C71" s="70" t="n">
+        <v>191</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="71" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="B72" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C72" s="72" t="n"/>
+      <c r="D72" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E71" s="72" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="72" t="inlineStr">
+      <c r="E72" s="71" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="71" t="inlineStr">
         <is>
           <t>TON</t>
         </is>
       </c>
-      <c r="B72" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C72" s="74" t="n"/>
-      <c r="D72" s="72" t="inlineStr">
+      <c r="B73" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C73" s="73" t="n"/>
+      <c r="D73" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E72" s="72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="72" t="inlineStr">
-        <is>
-          <t>TON</t>
-        </is>
-      </c>
-      <c r="B73" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C73" s="73" t="n"/>
-      <c r="D73" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E73" s="72" t="inlineStr"/>
+      <c r="E73" s="71" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5572,8 +5691,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C74" s="71" t="n">
-        <v>32174.288951</v>
+      <c r="C74" s="70" t="n">
+        <v>32097.231712</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -5593,8 +5712,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C75" s="71" t="n">
-        <v>32174.313939</v>
+      <c r="C75" s="70" t="n">
+        <v>32097.240025</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -5614,8 +5733,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C76" s="71" t="n">
-        <v>5678.20312</v>
+      <c r="C76" s="70" t="n">
+        <v>5638.408003</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -5639,7 +5758,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C77" s="71" t="n">
+      <c r="C77" s="70" t="n">
         <v>4797.537404</v>
       </c>
       <c r="D77" t="inlineStr">
@@ -5664,7 +5783,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C78" s="71" t="n">
+      <c r="C78" s="70" t="n">
         <v>3390556</v>
       </c>
       <c r="D78" t="inlineStr">
@@ -5689,7 +5808,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C79" s="71" t="n">
+      <c r="C79" s="70" t="n">
         <v>2916537</v>
       </c>
       <c r="D79" t="inlineStr">
@@ -5714,7 +5833,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C80" s="71" t="n">
+      <c r="C80" s="70" t="n">
         <v>348.971536</v>
       </c>
       <c r="D80" t="inlineStr">
@@ -5729,61 +5848,67 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="72" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>Tron</t>
         </is>
       </c>
-      <c r="B81" s="72" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C81" s="73" t="n"/>
-      <c r="D81" s="72" t="inlineStr">
+      <c r="C81" s="70" t="n">
+        <v>70</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="71" t="inlineStr">
+        <is>
+          <t>Tron</t>
+        </is>
+      </c>
+      <c r="B82" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C82" s="72" t="n"/>
+      <c r="D82" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E81" s="72" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="72" t="inlineStr">
+      <c r="E82" s="71" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="71" t="inlineStr">
         <is>
           <t>Tron</t>
         </is>
       </c>
-      <c r="B82" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C82" s="74" t="n"/>
-      <c r="D82" s="72" t="inlineStr">
+      <c r="B83" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C83" s="73" t="n"/>
+      <c r="D83" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E82" s="72" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="72" t="inlineStr">
-        <is>
-          <t>Tron</t>
-        </is>
-      </c>
-      <c r="B83" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C83" s="73" t="n"/>
-      <c r="D83" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E83" s="72" t="inlineStr"/>
+      <c r="E83" s="71" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5796,8 +5921,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C84" s="71" t="n">
-        <v>19075.239849</v>
+      <c r="C84" s="70" t="n">
+        <v>19786.883821</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -5817,8 +5942,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C85" s="71" t="n">
-        <v>81919.814663</v>
+      <c r="C85" s="70" t="n">
+        <v>84976.014364</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -5838,8 +5963,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C86" s="71" t="n">
-        <v>1190.593415</v>
+      <c r="C86" s="70" t="n">
+        <v>1171.952848</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -5863,7 +5988,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C87" s="71" t="n">
+      <c r="C87" s="70" t="n">
         <v>1672.171573</v>
       </c>
       <c r="D87" t="inlineStr">
@@ -5888,7 +6013,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C88" s="71" t="n">
+      <c r="C88" s="70" t="n">
         <v>86570</v>
       </c>
       <c r="D88" t="inlineStr">
@@ -5913,7 +6038,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C89" s="71" t="n">
+      <c r="C89" s="70" t="n">
         <v>64504</v>
       </c>
       <c r="D89" t="inlineStr">
@@ -5938,7 +6063,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C90" s="71" t="n">
+      <c r="C90" s="70" t="n">
         <v>910.588444</v>
       </c>
       <c r="D90" t="inlineStr">
@@ -5953,61 +6078,67 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="72" t="inlineStr">
+      <c r="A91" s="74" t="inlineStr">
         <is>
           <t>Hyperliquid</t>
         </is>
       </c>
-      <c r="B91" s="72" t="inlineStr">
+      <c r="B91" s="74" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C91" s="73" t="n"/>
-      <c r="D91" s="72" t="inlineStr">
+      <c r="C91" s="75" t="n">
+        <v>4</v>
+      </c>
+      <c r="D91" s="74" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E91" s="74" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0. ⚠ за 6 мес 24 → 4: скачок больше чем в 5 раз, часто это перепривязка общих репозиториев к сети, а не реальный приток разработчиков</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="71" t="inlineStr">
+        <is>
+          <t>Hyperliquid</t>
+        </is>
+      </c>
+      <c r="B92" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C92" s="72" t="n"/>
+      <c r="D92" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E91" s="72" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="72" t="inlineStr">
+      <c r="E92" s="71" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="71" t="inlineStr">
         <is>
           <t>Hyperliquid</t>
         </is>
       </c>
-      <c r="B92" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C92" s="74" t="n"/>
-      <c r="D92" s="72" t="inlineStr">
+      <c r="B93" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C93" s="73" t="n"/>
+      <c r="D93" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E92" s="72" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="72" t="inlineStr">
-        <is>
-          <t>Hyperliquid</t>
-        </is>
-      </c>
-      <c r="B93" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C93" s="73" t="n"/>
-      <c r="D93" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E93" s="72" t="inlineStr"/>
+      <c r="E93" s="71" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6020,8 +6151,8 @@
           <t>Капитализация, $ млн</t>
         </is>
       </c>
-      <c r="C94" s="71" t="n">
-        <v>328.245041</v>
+      <c r="C94" s="70" t="n">
+        <v>331.544745</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -6041,8 +6172,8 @@
           <t>FDV, $ млн</t>
         </is>
       </c>
-      <c r="C95" s="71" t="n">
-        <v>2794.774601</v>
+      <c r="C95" s="70" t="n">
+        <v>2822.869252</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -6062,8 +6193,8 @@
           <t>TVL сейчас, $ млн</t>
         </is>
       </c>
-      <c r="C96" s="71" t="n">
-        <v>1052.269901</v>
+      <c r="C96" s="70" t="n">
+        <v>1052.427495</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -6087,7 +6218,7 @@
           <t>TVL 6 мес назад, $ млн</t>
         </is>
       </c>
-      <c r="C97" s="71" t="n">
+      <c r="C97" s="70" t="n">
         <v>351.735124</v>
       </c>
       <c r="D97" t="inlineStr">
@@ -6112,7 +6243,7 @@
           <t>Активные адреса/день сейчас</t>
         </is>
       </c>
-      <c r="C98" s="71" t="n">
+      <c r="C98" s="70" t="n">
         <v>19904</v>
       </c>
       <c r="D98" t="inlineStr">
@@ -6137,7 +6268,7 @@
           <t>Активные адреса/день 6 мес назад</t>
         </is>
       </c>
-      <c r="C99" s="71" t="n">
+      <c r="C99" s="70" t="n">
         <v>13399</v>
       </c>
       <c r="D99" t="inlineStr">
@@ -6162,7 +6293,7 @@
           <t>Доход/комиссии за год, $ млн</t>
         </is>
       </c>
-      <c r="C100" s="71" t="n">
+      <c r="C100" s="70" t="n">
         <v>2.102234</v>
       </c>
       <c r="D100" t="inlineStr">
@@ -6177,61 +6308,67 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="72" t="inlineStr">
+      <c r="A101" t="inlineStr">
         <is>
           <t>Monad</t>
         </is>
       </c>
-      <c r="B101" s="72" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>Активных разработчиков/мес</t>
         </is>
       </c>
-      <c r="C101" s="73" t="n"/>
-      <c r="D101" s="72" t="inlineStr">
+      <c r="C101" s="70" t="n">
+        <v>75</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Open Dev Data</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>exclusive_devs за 28 дн до 2026-09-22. Source: Open Dev Data (opendevdata.org), CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="71" t="inlineStr">
+        <is>
+          <t>Monad</t>
+        </is>
+      </c>
+      <c r="B102" s="71" t="inlineStr">
+        <is>
+          <t>Разлок за 6 мес, % предложения</t>
+        </is>
+      </c>
+      <c r="C102" s="72" t="n"/>
+      <c r="D102" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E101" s="72" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="72" t="inlineStr">
+      <c r="E102" s="71" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="71" t="inlineStr">
         <is>
           <t>Monad</t>
         </is>
       </c>
-      <c r="B102" s="72" t="inlineStr">
-        <is>
-          <t>Разлок за 6 мес, % предложения</t>
-        </is>
-      </c>
-      <c r="C102" s="74" t="n"/>
-      <c r="D102" s="72" t="inlineStr">
+      <c r="B103" s="71" t="inlineStr">
+        <is>
+          <t>Инвесторы и команда, 1–5</t>
+        </is>
+      </c>
+      <c r="C103" s="73" t="n"/>
+      <c r="D103" s="71" t="inlineStr">
         <is>
           <t>нет данных — заполнить вручную</t>
         </is>
       </c>
-      <c r="E102" s="72" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="72" t="inlineStr">
-        <is>
-          <t>Monad</t>
-        </is>
-      </c>
-      <c r="B103" s="72" t="inlineStr">
-        <is>
-          <t>Инвесторы и команда, 1–5</t>
-        </is>
-      </c>
-      <c r="C103" s="73" t="n"/>
-      <c r="D103" s="72" t="inlineStr">
-        <is>
-          <t>нет данных — заполнить вручную</t>
-        </is>
-      </c>
-      <c r="E103" s="72" t="inlineStr"/>
+      <c r="E103" s="71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>